<commit_message>
used: finish lp bot
</commit_message>
<xml_diff>
--- a/08 - Excels/Open-LPs.xlsx
+++ b/08 - Excels/Open-LPs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\08 - Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30092D8E-7503-4129-8B97-BD2E0B0D8606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE4B84F1-AECA-464C-952B-21D61A76026F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$B$313</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$B$231</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="233">
   <si>
     <t>LP</t>
   </si>
@@ -67,111 +67,21 @@
     <t>LP-050565</t>
   </si>
   <si>
-    <t>LP-050631</t>
-  </si>
-  <si>
-    <t>LP-050632</t>
-  </si>
-  <si>
-    <t>LP-050633</t>
-  </si>
-  <si>
-    <t>LP-050635</t>
-  </si>
-  <si>
-    <t>LP-050827</t>
-  </si>
-  <si>
-    <t>LP-050839</t>
-  </si>
-  <si>
-    <t>LP-050858</t>
-  </si>
-  <si>
-    <t>LP-050859</t>
-  </si>
-  <si>
-    <t>LP-050873</t>
-  </si>
-  <si>
-    <t>LP-050929</t>
-  </si>
-  <si>
-    <t>LP-050956</t>
-  </si>
-  <si>
     <t>LP-050958</t>
   </si>
   <si>
-    <t>LP-050986</t>
-  </si>
-  <si>
-    <t>LP-051060</t>
-  </si>
-  <si>
-    <t>LP-051094</t>
-  </si>
-  <si>
-    <t>LP-051112</t>
-  </si>
-  <si>
-    <t>LP-051163</t>
-  </si>
-  <si>
-    <t>LP-051230</t>
-  </si>
-  <si>
-    <t>LP-051231</t>
-  </si>
-  <si>
-    <t>LP-051270</t>
-  </si>
-  <si>
-    <t>LP-051357</t>
-  </si>
-  <si>
-    <t>LP-051400</t>
-  </si>
-  <si>
-    <t>LP-051406</t>
-  </si>
-  <si>
-    <t>LP-051455</t>
-  </si>
-  <si>
-    <t>LP-051456</t>
-  </si>
-  <si>
-    <t>LP-051484</t>
+    <t>Compromisso pendente!</t>
   </si>
   <si>
     <t>LP-051570</t>
   </si>
   <si>
-    <t>LP-051592</t>
-  </si>
-  <si>
     <t>LP-051629</t>
   </si>
   <si>
-    <t>LP-051662</t>
-  </si>
-  <si>
-    <t>LP-051666</t>
-  </si>
-  <si>
-    <t>LP-051667</t>
-  </si>
-  <si>
     <t>LP-051684</t>
   </si>
   <si>
-    <t>LP-051747</t>
-  </si>
-  <si>
-    <t>LP-051844</t>
-  </si>
-  <si>
     <t>LP-051845</t>
   </si>
   <si>
@@ -181,175 +91,25 @@
     <t>LP-051847</t>
   </si>
   <si>
-    <t>LP-051855</t>
-  </si>
-  <si>
-    <t>LP-051857</t>
-  </si>
-  <si>
     <t>LP-051859</t>
   </si>
   <si>
-    <t>LP-051861</t>
-  </si>
-  <si>
     <t>LP-051865</t>
   </si>
   <si>
     <t>LP-051866</t>
   </si>
   <si>
-    <t>LP-051871</t>
-  </si>
-  <si>
-    <t>LP-051901</t>
-  </si>
-  <si>
-    <t>LP-051919</t>
-  </si>
-  <si>
     <t>LP-051931</t>
   </si>
   <si>
-    <t>LP-052006</t>
-  </si>
-  <si>
-    <t>LP-052007</t>
-  </si>
-  <si>
-    <t>LP-052019</t>
-  </si>
-  <si>
-    <t>LP-052021</t>
-  </si>
-  <si>
-    <t>LP-052083</t>
-  </si>
-  <si>
-    <t>LP-052086</t>
-  </si>
-  <si>
-    <t>LP-052094</t>
-  </si>
-  <si>
-    <t>LP-052095</t>
-  </si>
-  <si>
-    <t>LP-052166</t>
-  </si>
-  <si>
-    <t>LP-052197</t>
-  </si>
-  <si>
-    <t>LP-052211</t>
-  </si>
-  <si>
-    <t>LP-052295</t>
-  </si>
-  <si>
-    <t>LP-052299</t>
-  </si>
-  <si>
-    <t>LP-033611</t>
-  </si>
-  <si>
-    <t>LP-040735</t>
-  </si>
-  <si>
-    <t>LP-043162</t>
-  </si>
-  <si>
-    <t>LP-043280</t>
-  </si>
-  <si>
-    <t>LP-043975</t>
-  </si>
-  <si>
-    <t>LP-044234</t>
-  </si>
-  <si>
-    <t>LP-045835</t>
-  </si>
-  <si>
-    <t>LP-045874</t>
-  </si>
-  <si>
-    <t>LP-045877</t>
-  </si>
-  <si>
     <t>LP-046519</t>
   </si>
   <si>
-    <t>LP-046966</t>
-  </si>
-  <si>
-    <t>LP-047977</t>
-  </si>
-  <si>
-    <t>LP-047988</t>
-  </si>
-  <si>
-    <t>LP-048161</t>
-  </si>
-  <si>
-    <t>LP-048171</t>
-  </si>
-  <si>
-    <t>LP-048177</t>
-  </si>
-  <si>
-    <t>LP-048357</t>
-  </si>
-  <si>
-    <t>LP-048362</t>
-  </si>
-  <si>
-    <t>LP-049234</t>
-  </si>
-  <si>
-    <t>LP-049329</t>
-  </si>
-  <si>
-    <t>LP-049973</t>
-  </si>
-  <si>
-    <t>LP-050406</t>
-  </si>
-  <si>
-    <t>LP-050453</t>
-  </si>
-  <si>
-    <t>LP-050457</t>
-  </si>
-  <si>
-    <t>LP-050517</t>
-  </si>
-  <si>
     <t>LP-050538</t>
   </si>
   <si>
     <t>LP-050608</t>
-  </si>
-  <si>
-    <t>LP-050765</t>
-  </si>
-  <si>
-    <t>LP-050766</t>
-  </si>
-  <si>
-    <t>LP-050782</t>
-  </si>
-  <si>
-    <t>LP-050837</t>
-  </si>
-  <si>
-    <t>LP-050860</t>
-  </si>
-  <si>
-    <t>LP-050868</t>
-  </si>
-  <si>
-    <t>LP-050869</t>
   </si>
   <si>
     <t>LP-050918</t>
@@ -1324,7 +1084,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B313"/>
+  <dimension ref="A1:B231"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -1407,850 +1167,898 @@
       <c r="A10" t="s">
         <v>11</v>
       </c>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="B14" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+      <c r="B16" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="B17" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="B18" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="B19" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="B20" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="B21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+      <c r="B22" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="B23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="B24" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="B25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="150" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="169" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="170" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="172" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="173" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="174" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="175" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="176" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="177" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="178" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>179</v>
+        <v>26</v>
       </c>
     </row>
     <row r="179" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="180" spans="1:1" x14ac:dyDescent="0.25">
@@ -2511,416 +2319,6 @@
     <row r="231" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>232</v>
-      </c>
-    </row>
-    <row r="232" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A232" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="233" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A233" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="234" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A234" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="235" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A235" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="236" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A236" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="237" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A237" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="238" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A238" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="239" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A239" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="240" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A240" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="241" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A241" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="242" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A242" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="243" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A243" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="244" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A244" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="245" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A245" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="246" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A246" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="247" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A247" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="248" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A248" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="249" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A249" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="250" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A250" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="251" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A251" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="252" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A252" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="253" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A253" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="254" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A254" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="255" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A255" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="256" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A256" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="257" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A257" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="258" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A258" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="259" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A259" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="260" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A260" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="261" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A261" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="262" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A262" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="263" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A263" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="264" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A264" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="265" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A265" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="266" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A266" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="267" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A267" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="268" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A268" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="269" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A269" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="270" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A270" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="271" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A271" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="272" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A272" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="273" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A273" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="274" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A274" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="275" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A275" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="276" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A276" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="277" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A277" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="278" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A278" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="279" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A279" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="280" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A280" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="281" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A281" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="282" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A282" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="283" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A283" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="284" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A284" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="285" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A285" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="286" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A286" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="287" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A287" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="288" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A288" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="289" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A289" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="290" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A290" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="291" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A291" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="292" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A292" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="293" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A293" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="294" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A294" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="295" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A295" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="296" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A296" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="297" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A297" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="298" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A298" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="299" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A299" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="300" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A300" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="301" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A301" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="302" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A302" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="303" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A303" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="304" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A304" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="305" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A305" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="306" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A306" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="307" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A307" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="308" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A308" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="309" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A309" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="310" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A310" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="311" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A311" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="312" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A312" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="313" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A313" t="s">
-        <v>312</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: finish lp bot
</commit_message>
<xml_diff>
--- a/08 - Excels/Open-LPs.xlsx
+++ b/08 - Excels/Open-LPs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\08 - Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E7C55ED-4680-4AB8-8F0C-53E597EE62F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AD0DCE1-A742-4978-BC15-3BD15206B2E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$B$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$B$40</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="41">
   <si>
     <t>LP</t>
   </si>
@@ -37,18 +37,9 @@
     <t>Possui linhas de compra e apontamento!</t>
   </si>
   <si>
-    <t>LP-051263</t>
-  </si>
-  <si>
-    <t>LP-051320</t>
-  </si>
-  <si>
     <t>LP-051497</t>
   </si>
   <si>
-    <t>LP-051624</t>
-  </si>
-  <si>
     <t>LP-051680</t>
   </si>
   <si>
@@ -121,121 +112,13 @@
     <t>LP-052018</t>
   </si>
   <si>
-    <t>LP-052028</t>
-  </si>
-  <si>
-    <t>LP-052029</t>
-  </si>
-  <si>
-    <t>LP-052030</t>
-  </si>
-  <si>
-    <t>LP-052031</t>
-  </si>
-  <si>
-    <t>LP-052032</t>
-  </si>
-  <si>
-    <t>LP-052061</t>
-  </si>
-  <si>
-    <t>LP-052093</t>
-  </si>
-  <si>
-    <t>LP-052108</t>
-  </si>
-  <si>
-    <t>LP-052109</t>
-  </si>
-  <si>
-    <t>LP-052136</t>
-  </si>
-  <si>
-    <t>LP-052148</t>
-  </si>
-  <si>
     <t>LP-052153</t>
   </si>
   <si>
-    <t>LP-052152</t>
-  </si>
-  <si>
-    <t>LP-052212</t>
-  </si>
-  <si>
-    <t>LP-052214</t>
-  </si>
-  <si>
-    <t>LP-052262</t>
-  </si>
-  <si>
-    <t>LP-052480</t>
-  </si>
-  <si>
-    <t>LP-052487</t>
-  </si>
-  <si>
-    <t>LP-052504</t>
-  </si>
-  <si>
-    <t>LP-052508</t>
-  </si>
-  <si>
-    <t>LP-052509</t>
-  </si>
-  <si>
-    <t>LP-052513</t>
-  </si>
-  <si>
-    <t>LP-052514</t>
-  </si>
-  <si>
-    <t>LP-052572</t>
-  </si>
-  <si>
-    <t>LP-052608</t>
-  </si>
-  <si>
-    <t>LP-052628</t>
-  </si>
-  <si>
-    <t>LP-052688</t>
-  </si>
-  <si>
-    <t>LP-052782</t>
-  </si>
-  <si>
-    <t>LP-052861</t>
-  </si>
-  <si>
-    <t>LP-052986</t>
-  </si>
-  <si>
-    <t>LP-045478</t>
-  </si>
-  <si>
-    <t>LP-045674</t>
-  </si>
-  <si>
-    <t>LP-048423</t>
-  </si>
-  <si>
     <t>LP-048713</t>
   </si>
   <si>
     <t>LP-048714</t>
-  </si>
-  <si>
-    <t>LP-049936</t>
-  </si>
-  <si>
-    <t>LP-050094</t>
-  </si>
-  <si>
-    <t>LP-050096</t>
-  </si>
-  <si>
-    <t>LP-050127</t>
   </si>
   <si>
     <t>LP-050143</t>
@@ -625,7 +508,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B80"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -652,148 +535,235 @@
       <c r="A3" t="s">
         <v>4</v>
       </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
+      <c r="B9" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
+      <c r="B13" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>15</v>
       </c>
+      <c r="B14" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="B17" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>32</v>
       </c>
@@ -836,206 +806,6 @@
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
-        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: we are back
</commit_message>
<xml_diff>
--- a/08 - Excels/Open-LPs.xlsx
+++ b/08 - Excels/Open-LPs.xlsx
@@ -8,22 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\08 - Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62EF6994-470C-4D2B-9C25-7F6878C8DF70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2E09CB-A927-44A1-987F-159CB72691AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$B$40</definedName>
-  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="72">
   <si>
     <t>LP</t>
   </si>
@@ -31,60 +28,12 @@
     <t>Status</t>
   </si>
   <si>
-    <t>LP-007876</t>
-  </si>
-  <si>
-    <t>LP-008079</t>
-  </si>
-  <si>
-    <t>LP-008046</t>
-  </si>
-  <si>
-    <t>LP-008767</t>
-  </si>
-  <si>
-    <t>LP-008769</t>
-  </si>
-  <si>
-    <t>LP-010221</t>
-  </si>
-  <si>
-    <t>LP-011252</t>
-  </si>
-  <si>
-    <t>LP-010943</t>
-  </si>
-  <si>
-    <t>LP-010944</t>
-  </si>
-  <si>
-    <t>LP-011239</t>
-  </si>
-  <si>
-    <t>LP-011914</t>
-  </si>
-  <si>
-    <t>LP-011915</t>
-  </si>
-  <si>
-    <t>LP-011916</t>
-  </si>
-  <si>
-    <t>LP-011917</t>
-  </si>
-  <si>
-    <t>LP-011691</t>
-  </si>
-  <si>
-    <t>LP-011958</t>
-  </si>
-  <si>
-    <t>LP-011949</t>
-  </si>
-  <si>
     <t>LP-012703</t>
   </si>
   <si>
+    <t>Compromisso pendente!</t>
+  </si>
+  <si>
     <t>LP-012547</t>
   </si>
   <si>
@@ -94,184 +43,10 @@
     <t>LP-012548</t>
   </si>
   <si>
-    <t>LP-013161</t>
-  </si>
-  <si>
-    <t>LP-013337</t>
-  </si>
-  <si>
-    <t>LP-013444</t>
-  </si>
-  <si>
-    <t>LP-014697</t>
-  </si>
-  <si>
-    <t>LP-016075</t>
-  </si>
-  <si>
-    <t>LP-016199</t>
-  </si>
-  <si>
-    <t>LP-017180</t>
-  </si>
-  <si>
-    <t>LP-017093</t>
-  </si>
-  <si>
-    <t>LP-017034</t>
-  </si>
-  <si>
-    <t>LP-017035</t>
-  </si>
-  <si>
-    <t>LP-018651</t>
-  </si>
-  <si>
-    <t>LP-019026</t>
-  </si>
-  <si>
-    <t>LP-018908</t>
-  </si>
-  <si>
-    <t>LP-019151</t>
-  </si>
-  <si>
-    <t>LP-019500</t>
-  </si>
-  <si>
-    <t>LP-019480</t>
-  </si>
-  <si>
-    <t>LP-019552</t>
-  </si>
-  <si>
-    <t>LP-020403</t>
-  </si>
-  <si>
-    <t>LP-020609</t>
-  </si>
-  <si>
-    <t>LP-022028</t>
-  </si>
-  <si>
-    <t>LP-030877</t>
-  </si>
-  <si>
-    <t>LP-031038</t>
-  </si>
-  <si>
-    <t>LP-026526</t>
-  </si>
-  <si>
-    <t>LP-026366</t>
-  </si>
-  <si>
-    <t>LP-026553</t>
-  </si>
-  <si>
-    <t>LP-027839</t>
-  </si>
-  <si>
-    <t>LP-027036</t>
-  </si>
-  <si>
-    <t>LP-027840</t>
-  </si>
-  <si>
-    <t>LP-027818</t>
-  </si>
-  <si>
-    <t>LP-027830</t>
-  </si>
-  <si>
-    <t>LP-028616</t>
-  </si>
-  <si>
-    <t>LP-028618</t>
-  </si>
-  <si>
-    <t>LP-028615</t>
-  </si>
-  <si>
-    <t>LP-028617</t>
-  </si>
-  <si>
-    <t>LP-029253</t>
-  </si>
-  <si>
-    <t>LP-029890</t>
-  </si>
-  <si>
-    <t>LP-029920</t>
-  </si>
-  <si>
-    <t>LP-030878</t>
-  </si>
-  <si>
-    <t>LP-030448</t>
-  </si>
-  <si>
-    <t>LP-031089</t>
-  </si>
-  <si>
-    <t>LP-030860</t>
-  </si>
-  <si>
-    <t>LP-030801</t>
-  </si>
-  <si>
-    <t>LP-031399</t>
-  </si>
-  <si>
-    <t>LP-031498</t>
-  </si>
-  <si>
-    <t>LP-032265</t>
-  </si>
-  <si>
-    <t>LP-032339</t>
-  </si>
-  <si>
-    <t>LP-032473</t>
-  </si>
-  <si>
-    <t>LP-033819</t>
-  </si>
-  <si>
     <t>LP-033921</t>
   </si>
   <si>
-    <t>LP-033202</t>
-  </si>
-  <si>
-    <t>LP-033817</t>
-  </si>
-  <si>
-    <t>LP-033926</t>
-  </si>
-  <si>
     <t>LP-034178</t>
-  </si>
-  <si>
-    <t>LP-033959</t>
-  </si>
-  <si>
-    <t>LP-033960</t>
-  </si>
-  <si>
-    <t>LP-035078</t>
-  </si>
-  <si>
-    <t>LP-035156</t>
-  </si>
-  <si>
-    <t>LP-035157</t>
-  </si>
-  <si>
-    <t>LP-037846</t>
-  </si>
-  <si>
-    <t>LP-035933</t>
   </si>
   <si>
     <t>LP-037048</t>
@@ -479,7 +254,6 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -824,11 +598,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B145"/>
+  <dimension ref="A1:B70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -843,720 +617,363 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
         <v>71</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A129" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A130" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A131" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A132" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A133" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A135" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A136" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A137" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A138" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A139" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A140" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A141" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A142" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A143" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A144" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A145" t="s">
-        <v>145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
used: finish LP and OM bot
</commit_message>
<xml_diff>
--- a/08 - Excels/Open-LPs.xlsx
+++ b/08 - Excels/Open-LPs.xlsx
@@ -8,19 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\feb3ct\Desktop\PyAutomateSAP\08 - Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACB29296-69C2-4EF9-8881-3AD34CD8C766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{527D5B02-7FDC-4CCC-97F3-9598A9D6481C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$B$22</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="24">
   <si>
     <t>LP</t>
   </si>
@@ -28,96 +31,18 @@
     <t>Status</t>
   </si>
   <si>
-    <t>LP-051369</t>
-  </si>
-  <si>
-    <t>LP-051388</t>
-  </si>
-  <si>
-    <t>LP-051391</t>
-  </si>
-  <si>
-    <t>LP-051395</t>
-  </si>
-  <si>
-    <t>LP-051425</t>
-  </si>
-  <si>
-    <t>LP-051431</t>
-  </si>
-  <si>
-    <t>LP-051432</t>
-  </si>
-  <si>
-    <t>LP-051434</t>
-  </si>
-  <si>
-    <t>LP-051448</t>
-  </si>
-  <si>
-    <t>LP-051449</t>
-  </si>
-  <si>
-    <t>LP-051519</t>
-  </si>
-  <si>
-    <t>LP-051540</t>
-  </si>
-  <si>
-    <t>LP-051541</t>
-  </si>
-  <si>
-    <t>LP-051543</t>
-  </si>
-  <si>
-    <t>LP-051705</t>
-  </si>
-  <si>
-    <t>LP-051712</t>
-  </si>
-  <si>
-    <t>LP-051716</t>
-  </si>
-  <si>
-    <t>LP-052122</t>
-  </si>
-  <si>
-    <t>LP-052138</t>
-  </si>
-  <si>
-    <t>LP-052141</t>
-  </si>
-  <si>
-    <t>LP-052160</t>
-  </si>
-  <si>
-    <t>LP-052199</t>
-  </si>
-  <si>
-    <t>LP-052308</t>
-  </si>
-  <si>
     <t>LP-052309</t>
   </si>
   <si>
+    <t>Compromisso pendente!</t>
+  </si>
+  <si>
     <t>LP-052311</t>
   </si>
   <si>
     <t>LP-052312</t>
   </si>
   <si>
-    <t>LP-052326</t>
-  </si>
-  <si>
-    <t>LP-052372</t>
-  </si>
-  <si>
-    <t>LP-052381</t>
-  </si>
-  <si>
-    <t>LP-052386</t>
-  </si>
-  <si>
     <t>LP-052400</t>
   </si>
   <si>
@@ -167,12 +92,6 @@
   </si>
   <si>
     <t>LP-052773</t>
-  </si>
-  <si>
-    <t>LP-052978</t>
-  </si>
-  <si>
-    <t>LP-053040</t>
   </si>
   <si>
     <t>LP-053105</t>
@@ -538,11 +457,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -557,250 +476,168 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="B9" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="B14" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="B16" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+      <c r="B17" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="B18" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="B19" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="B20" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="B21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>51</v>
+      <c r="B22" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>